<commit_message>
Excel add-in + richer snapshot tracking; grok-bot prompt for project collab
- Track fonts, borders, alignment, layout, merges, freeze, hidden sheets
- Local Bit agent: data dir, version graph, pick-folder
- Sideload Excel task pane: save version, scenarios, history, graph
- Docs for add-in, repo map, functionality
- Next: SharePoint as project remote, append-only store, promote-to-Main (GROK-BOT-PROMPT.md)
</commit_message>
<xml_diff>
--- a/fixtures/sample-budget.xlsx
+++ b/fixtures/sample-budget.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Line Item</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t>Tax</t>
+  </si>
+  <si>
+    <t>Source notes</t>
   </si>
   <si>
     <t>Tax Rate</t>
@@ -54,7 +57,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -68,6 +71,10 @@
     </font>
     <font>
       <b/>
+      <u/>
+    </font>
+    <font>
+      <b/>
     </font>
     <font>
       <b/>
@@ -75,12 +82,17 @@
     </font>
     <font>
       <color rgb="FFFF0000"/>
+      <strike/>
     </font>
     <font>
       <i/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -99,11 +111,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF4B183"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -111,22 +128,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,82 +507,100 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <sheetPr>
+    <tabColor rgb="FF4472C4"/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="4">
         <v>100000</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="5">
         <v>110000</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="6">
         <f>B2+C2</f>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" hidden="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>40000</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="5">
         <v>44000</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="5">
         <f>B3+C3</f>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="8">
         <f>B2-B3</f>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="8">
         <f>C2-C3</f>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="8">
         <f>D2-D3</f>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <f>Assumptions!B1</f>
       </c>
+      <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="11">
         <f>B4*B6</f>
       </c>
     </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="12"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A8:B8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -551,21 +610,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="3" max="3" width="12" hidden="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="9">
+      <c r="A1" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="14">
         <v>0.21</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>10</v>
+      <c r="A2" s="15" t="s">
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>